<commit_message>
test: regenerate the files for checking in Excel, add a volatile spill that shrinks
</commit_message>
<xml_diff>
--- a/tools/excel-oracle/writer-check/spill-blocked.xlsx
+++ b/tools/excel-oracle/writer-check/spill-blocked.xlsx
@@ -54,11 +54,18 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="1">
+  <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
         </ext>
       </extLst>
     </bk>
@@ -68,9 +75,12 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="1">
+  <valueMetadata count="2">
     <bk>
       <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -240,23 +250,31 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
   <rv s="0">
     <v>1</v>
     <v>8</v>
     <v>9</v>
     <v>1</v>
   </rv>
+  <rv s="1">
+    <v>8</v>
+    <v>1</v>
+  </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
   <s t="_error">
     <k n="colOffset" t="i"/>
     <k n="errorType" t="i"/>
     <k n="rwOffset" t="i"/>
     <k n="subType" t="i"/>
+  </s>
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="propagated" t="b"/>
   </s>
 </rvStructures>
 </file>
@@ -595,9 +613,9 @@
       <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="3" cm="1" t="e">
+      <c r="F3" s="3" cm="1" t="e" vm="2">
         <f t="array" ref="F3">_xlfn.TAKE(_xlfn.ANCHORARRAY(A3),3,1)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="G3" t="s">
         <v>3</v>
@@ -656,9 +674,9 @@
       <c r="B12" s="3"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" t="e">
+      <c r="A14" t="e" vm="2">
         <f>SUM(_xlfn.ANCHORARRAY(A3))</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="B14" t="s">
         <v>2</v>
@@ -667,15 +685,15 @@
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="3" cm="1">
         <f t="array" aca="1" ref="A19:C21" ca="1">_xlfn.RANDARRAY(3,3, 0, 100,TRUE)</f>
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="B19" s="3">
         <f ca="1"/>
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="C19" s="3">
         <f ca="1"/>
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E19" t="s">
         <v>4</v>
@@ -684,29 +702,29 @@
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <f ca="1"/>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B20" s="3">
         <f ca="1"/>
-        <v>31</v>
+        <v>90</v>
       </c>
       <c r="C20" s="3">
         <f ca="1"/>
-        <v>11</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <f ca="1"/>
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B21" s="3">
         <f ca="1"/>
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="C21" s="3">
         <f ca="1"/>
-        <v>24</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>